<commit_message>
docs(historias): alinea las HU con la numeracion de Santiago (RQF-13..26)
- HU-54..58 apuntan a los codigos nuevos: HU-54 RQF-13, HU-55 RQF-14,
  HU-56 RQF-16 y RQF-19, HU-57 y HU-58 RQF-15 (HU-58 ahora incluye
  hitos y retos activos).
- HU-34 cubre tambien RQF-24 (listado de ingresos).
- Nuevas HU-59..66 para RQF-17, 18, 20, 21, 22, 23, 25 y 26, con 5
  criterios de aceptacion coherentes con el docx de docs/.
- La lista de prioridad cubre las 66 HU. Las 26 RF tienen historia.
</commit_message>
<xml_diff>
--- a/Documentación/Plantilla historias de usuario.xlsx
+++ b/Documentación/Plantilla historias de usuario.xlsx
@@ -4492,7 +4492,7 @@
       </c>
       <c r="G202" s="31" t="inlineStr">
         <is>
-          <t>Operación READ en tiempo real del módulo Check-in (RQF-05 y RQF-07).</t>
+          <t>Operación READ en tiempo real del módulo Check-in (RQF-05, RQF-07 y RQF-24).</t>
         </is>
       </c>
     </row>
@@ -6394,7 +6394,7 @@
       </c>
       <c r="G322" s="31" t="inlineStr">
         <is>
-          <t>Operación CREATE del envío de contrato en el módulo Gestión de Miembros (RQF-13). Depende de RQF-03.</t>
+          <t>Operación CREATE del envío de contrato en el módulo Contratos (RQF-13). Depende de RQF-03.</t>
         </is>
       </c>
     </row>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="G334" s="31" t="inlineStr">
         <is>
-          <t>Operación CREATE de gimnasio y cuenta dueño en el módulo Suscripción SaaS (RQF-15). Relacionado con RQNF-05.</t>
+          <t>Operación CREATE de gimnasio y cuenta dueño, con prueba gratuita (RQF-16 y RQF-19). Relacionado con RQNF-05.</t>
         </is>
       </c>
     </row>
@@ -6724,7 +6724,7 @@
       </c>
       <c r="G340" s="26" t="inlineStr">
         <is>
-          <t>Operación CREATE de sesión del miembro en el módulo App Móvil del Miembro (RQF-16). Depende de RQF-03.</t>
+          <t>Operación CREATE de sesión del miembro en el módulo App del miembro (RQF-15). Depende de RQF-03.</t>
         </is>
       </c>
     </row>
@@ -6809,12 +6809,12 @@
       <c r="A346" s="7" t="n"/>
       <c r="B346" s="27" t="inlineStr">
         <is>
-          <t>HU-58: Consultar QR, plan y asistencia desde la app móvil</t>
+          <t>HU-58: Consultar QR, plan, asistencia y logros desde la app móvil</t>
         </is>
       </c>
       <c r="C346" s="29" t="inlineStr">
         <is>
-          <t>Como miembro, quiero ver en la app mi código QR, mi plan vigente y mi historial de asistencia, para que pueda ingresar al gimnasio y conocer el estado de mi membresía.</t>
+          <t>Como miembro, quiero ver en la app mi código QR, mi plan vigente, mi historial de asistencia, mis hitos y los retos activos, para que pueda ingresar al gimnasio y seguir mi progreso.</t>
         </is>
       </c>
       <c r="D346" s="15" t="inlineStr">
@@ -6834,7 +6834,7 @@
       </c>
       <c r="G346" s="31" t="inlineStr">
         <is>
-          <t>Operación READ del módulo App Móvil del Miembro (RQF-16). Depende de HU-57.</t>
+          <t>Operación READ del módulo App del miembro (RQF-15). Depende de HU-57.</t>
         </is>
       </c>
     </row>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="E349" s="31" t="inlineStr">
         <is>
-          <t>El miembro puede actualizar su teléfono, su correo y su contacto de emergencia.</t>
+          <t>La app muestra los hitos logrados y los retos activos del gimnasio con el avance del miembro.</t>
         </is>
       </c>
       <c r="F349" s="23" t="n"/>
@@ -6917,195 +6917,883 @@
     </row>
     <row r="352" ht="18" customHeight="1">
       <c r="A352" s="7" t="n"/>
-      <c r="D352" s="17" t="n"/>
+      <c r="B352" s="25" t="inlineStr">
+        <is>
+          <t>HU-59: Recuperar la contraseña con un código enviado al correo</t>
+        </is>
+      </c>
+      <c r="C352" s="28" t="inlineStr">
+        <is>
+          <t>Como miembro del personal, quiero recuperar mi contraseña con un código que llega a mi correo, para que pueda volver a entrar al sistema sin pedir ayuda al administrador.</t>
+        </is>
+      </c>
+      <c r="D352" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E352" s="26" t="inlineStr">
+        <is>
+          <t>Desde la pantalla de inicio de sesión puedo solicitar la recuperación indicando mi correo.</t>
+        </is>
+      </c>
+      <c r="F352" s="30" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G352" s="26" t="inlineStr">
+        <is>
+          <t>Operación UPDATE de credenciales en el módulo Gestión de Usuarios (RQF-17). Relacionado con RQNF-09.</t>
+        </is>
+      </c>
     </row>
     <row r="353" ht="18" customHeight="1">
       <c r="A353" s="7" t="n"/>
-      <c r="D353" s="17" t="n"/>
+      <c r="B353" s="23" t="n"/>
+      <c r="C353" s="23" t="n"/>
+      <c r="D353" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E353" s="26" t="inlineStr">
+        <is>
+          <t>El sistema envía al correo un código de 6 dígitos válido por 15 minutos.</t>
+        </is>
+      </c>
+      <c r="F353" s="23" t="n"/>
+      <c r="G353" s="23" t="n"/>
     </row>
     <row r="354" ht="18" customHeight="1">
       <c r="A354" s="7" t="n"/>
-      <c r="D354" s="17" t="n"/>
+      <c r="B354" s="23" t="n"/>
+      <c r="C354" s="23" t="n"/>
+      <c r="D354" s="11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E354" s="26" t="inlineStr">
+        <is>
+          <t>Solo con un código válido y vigente puedo definir la nueva contraseña.</t>
+        </is>
+      </c>
+      <c r="F354" s="23" t="n"/>
+      <c r="G354" s="23" t="n"/>
     </row>
     <row r="355" ht="18" customHeight="1">
       <c r="A355" s="7" t="n"/>
-      <c r="D355" s="17" t="n"/>
+      <c r="B355" s="23" t="n"/>
+      <c r="C355" s="23" t="n"/>
+      <c r="D355" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E355" s="26" t="inlineStr">
+        <is>
+          <t>La nueva contraseña se guarda cifrada con bcrypt y con ella puedo iniciar sesión.</t>
+        </is>
+      </c>
+      <c r="F355" s="23" t="n"/>
+      <c r="G355" s="23" t="n"/>
     </row>
     <row r="356" ht="18" customHeight="1">
       <c r="A356" s="7" t="n"/>
-      <c r="D356" s="17" t="n"/>
+      <c r="B356" s="24" t="n"/>
+      <c r="C356" s="24" t="n"/>
+      <c r="D356" s="11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E356" s="26" t="inlineStr">
+        <is>
+          <t>El sistema limita las solicitudes de recuperación a 3 por minuto.</t>
+        </is>
+      </c>
+      <c r="F356" s="24" t="n"/>
+      <c r="G356" s="24" t="n"/>
     </row>
     <row r="357" ht="18" customHeight="1">
       <c r="A357" s="7" t="n"/>
-      <c r="D357" s="17" t="n"/>
+      <c r="B357" s="34" t="n"/>
+      <c r="C357" s="34" t="n"/>
+      <c r="D357" s="35" t="n"/>
+      <c r="E357" s="34" t="n"/>
+      <c r="F357" s="34" t="n"/>
+      <c r="G357" s="34" t="n"/>
     </row>
     <row r="358" ht="18" customHeight="1">
       <c r="A358" s="7" t="n"/>
-      <c r="D358" s="17" t="n"/>
+      <c r="B358" s="27" t="inlineStr">
+        <is>
+          <t>HU-60: Exportar el listado de miembros activos a CSV</t>
+        </is>
+      </c>
+      <c r="C358" s="29" t="inlineStr">
+        <is>
+          <t>Como administrador, quiero descargar en CSV el listado de miembros activos con su membresía, para que pueda analizarlo o compartirlo en una hoja de cálculo.</t>
+        </is>
+      </c>
+      <c r="D358" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E358" s="31" t="inlineStr">
+        <is>
+          <t>El dashboard tiene un botón para descargar el archivo CSV.</t>
+        </is>
+      </c>
+      <c r="F358" s="22" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G358" s="31" t="inlineStr">
+        <is>
+          <t>Operación READ / exportación del módulo Dashboard (RQF-18).</t>
+        </is>
+      </c>
     </row>
     <row r="359" ht="18" customHeight="1">
       <c r="A359" s="7" t="n"/>
-      <c r="D359" s="17" t="n"/>
+      <c r="B359" s="23" t="n"/>
+      <c r="C359" s="23" t="n"/>
+      <c r="D359" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E359" s="31" t="inlineStr">
+        <is>
+          <t>El archivo incluye solo los miembros activos de mi gimnasio con documento, contacto, plan, fecha de fin y días restantes.</t>
+        </is>
+      </c>
+      <c r="F359" s="23" t="n"/>
+      <c r="G359" s="23" t="n"/>
     </row>
     <row r="360" ht="18" customHeight="1">
       <c r="A360" s="7" t="n"/>
-      <c r="D360" s="17" t="n"/>
+      <c r="B360" s="23" t="n"/>
+      <c r="C360" s="23" t="n"/>
+      <c r="D360" s="15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E360" s="31" t="inlineStr">
+        <is>
+          <t>El archivo se abre en Excel con tildes y eñes correctas (UTF-8 con BOM).</t>
+        </is>
+      </c>
+      <c r="F360" s="23" t="n"/>
+      <c r="G360" s="23" t="n"/>
     </row>
     <row r="361" ht="18" customHeight="1">
       <c r="A361" s="7" t="n"/>
-      <c r="D361" s="17" t="n"/>
+      <c r="B361" s="23" t="n"/>
+      <c r="C361" s="23" t="n"/>
+      <c r="D361" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E361" s="31" t="inlineStr">
+        <is>
+          <t>El nombre del archivo incluye la fecha de la descarga.</t>
+        </is>
+      </c>
+      <c r="F361" s="23" t="n"/>
+      <c r="G361" s="23" t="n"/>
     </row>
     <row r="362" ht="18" customHeight="1">
       <c r="A362" s="7" t="n"/>
-      <c r="D362" s="17" t="n"/>
+      <c r="B362" s="24" t="n"/>
+      <c r="C362" s="24" t="n"/>
+      <c r="D362" s="15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E362" s="31" t="inlineStr">
+        <is>
+          <t>Solo el rol Administrador puede descargarlo.</t>
+        </is>
+      </c>
+      <c r="F362" s="24" t="n"/>
+      <c r="G362" s="24" t="n"/>
     </row>
     <row r="363" ht="18" customHeight="1">
       <c r="A363" s="7" t="n"/>
-      <c r="D363" s="17" t="n"/>
+      <c r="B363" s="34" t="n"/>
+      <c r="C363" s="34" t="n"/>
+      <c r="D363" s="35" t="n"/>
+      <c r="E363" s="34" t="n"/>
+      <c r="F363" s="34" t="n"/>
+      <c r="G363" s="34" t="n"/>
     </row>
     <row r="364" ht="18" customHeight="1">
       <c r="A364" s="7" t="n"/>
-      <c r="D364" s="17" t="n"/>
+      <c r="B364" s="25" t="inlineStr">
+        <is>
+          <t>HU-61: Configurar precios de planes y recordatorios de cobro</t>
+        </is>
+      </c>
+      <c r="C364" s="28" t="inlineStr">
+        <is>
+          <t>Como administrador, quiero configurar el precio de cada tipo de plan y los recordatorios de cobro de mi gimnasio, para que los valores y los avisos correspondan a mi negocio.</t>
+        </is>
+      </c>
+      <c r="D364" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E364" s="26" t="inlineStr">
+        <is>
+          <t>Puedo definir el precio de los planes mensual, trimestral, semestral, anual, clase suelta e ilimitado.</t>
+        </is>
+      </c>
+      <c r="F364" s="30" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G364" s="26" t="inlineStr">
+        <is>
+          <t>Operación UPDATE de parámetros del gimnasio en el módulo Configuración (RQF-20). Relacionado con CU09.</t>
+        </is>
+      </c>
     </row>
     <row r="365" ht="18" customHeight="1">
       <c r="A365" s="7" t="n"/>
-      <c r="D365" s="17" t="n"/>
+      <c r="B365" s="23" t="n"/>
+      <c r="C365" s="23" t="n"/>
+      <c r="D365" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E365" s="26" t="inlineStr">
+        <is>
+          <t>Puedo activar o desactivar los recordatorios de cobro.</t>
+        </is>
+      </c>
+      <c r="F365" s="23" t="n"/>
+      <c r="G365" s="23" t="n"/>
     </row>
     <row r="366" ht="18" customHeight="1">
       <c r="A366" s="7" t="n"/>
-      <c r="D366" s="17" t="n"/>
+      <c r="B366" s="23" t="n"/>
+      <c r="C366" s="23" t="n"/>
+      <c r="D366" s="11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E366" s="26" t="inlineStr">
+        <is>
+          <t>Puedo definir con cuántos días de anticipación se avisa, entre 1 y 30.</t>
+        </is>
+      </c>
+      <c r="F366" s="23" t="n"/>
+      <c r="G366" s="23" t="n"/>
     </row>
     <row r="367" ht="18" customHeight="1">
       <c r="A367" s="7" t="n"/>
-      <c r="D367" s="17" t="n"/>
+      <c r="B367" s="23" t="n"/>
+      <c r="C367" s="23" t="n"/>
+      <c r="D367" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E367" s="26" t="inlineStr">
+        <is>
+          <t>El sistema rechaza precios negativos.</t>
+        </is>
+      </c>
+      <c r="F367" s="23" t="n"/>
+      <c r="G367" s="23" t="n"/>
     </row>
     <row r="368" ht="18" customHeight="1">
       <c r="A368" s="7" t="n"/>
-      <c r="D368" s="17" t="n"/>
+      <c r="B368" s="24" t="n"/>
+      <c r="C368" s="24" t="n"/>
+      <c r="D368" s="11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E368" s="26" t="inlineStr">
+        <is>
+          <t>Los avisos de cobro del centro de notificaciones usan la configuración guardada.</t>
+        </is>
+      </c>
+      <c r="F368" s="24" t="n"/>
+      <c r="G368" s="24" t="n"/>
     </row>
     <row r="369" ht="18" customHeight="1">
       <c r="A369" s="7" t="n"/>
-      <c r="D369" s="17" t="n"/>
+      <c r="B369" s="34" t="n"/>
+      <c r="C369" s="34" t="n"/>
+      <c r="D369" s="35" t="n"/>
+      <c r="E369" s="34" t="n"/>
+      <c r="F369" s="34" t="n"/>
+      <c r="G369" s="34" t="n"/>
     </row>
     <row r="370" ht="18" customHeight="1">
       <c r="A370" s="7" t="n"/>
-      <c r="D370" s="17" t="n"/>
+      <c r="B370" s="27" t="inlineStr">
+        <is>
+          <t>HU-62: Registrar el plan y el pago de un miembro</t>
+        </is>
+      </c>
+      <c r="C370" s="29" t="inlineStr">
+        <is>
+          <t>Como administrador o recepcionista, quiero registrar el plan contratado y el pago de cada miembro, para que pueda saber quién está al día y cuánto debe.</t>
+        </is>
+      </c>
+      <c r="D370" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E370" s="31" t="inlineStr">
+        <is>
+          <t>Al registrar o renovar un plan se guardan el tipo de plan y las fechas de inicio y fin.</t>
+        </is>
+      </c>
+      <c r="F370" s="22" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G370" s="31" t="inlineStr">
+        <is>
+          <t>Operación CREATE / UPDATE de plan y pago en el módulo Gestión de Miembros (RQF-21). Relacionado con CU08.</t>
+        </is>
+      </c>
     </row>
     <row r="371" ht="18" customHeight="1">
       <c r="A371" s="7" t="n"/>
-      <c r="D371" s="17" t="n"/>
+      <c r="B371" s="23" t="n"/>
+      <c r="C371" s="23" t="n"/>
+      <c r="D371" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E371" s="31" t="inlineStr">
+        <is>
+          <t>Se registran el valor total, el valor pagado y el método de pago (efectivo, transferencia, tarjeta, PSE, Nequi, Daviplata u otro).</t>
+        </is>
+      </c>
+      <c r="F371" s="23" t="n"/>
+      <c r="G371" s="23" t="n"/>
     </row>
     <row r="372" ht="18" customHeight="1">
       <c r="A372" s="7" t="n"/>
-      <c r="D372" s="17" t="n"/>
+      <c r="B372" s="23" t="n"/>
+      <c r="C372" s="23" t="n"/>
+      <c r="D372" s="15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E372" s="31" t="inlineStr">
+        <is>
+          <t>Si no se indica, el estado del pago (Pendiente, Parcial o Pagado) se calcula a partir de los valores.</t>
+        </is>
+      </c>
+      <c r="F372" s="23" t="n"/>
+      <c r="G372" s="23" t="n"/>
     </row>
     <row r="373" ht="18" customHeight="1">
       <c r="A373" s="7" t="n"/>
-      <c r="D373" s="17" t="n"/>
+      <c r="B373" s="23" t="n"/>
+      <c r="C373" s="23" t="n"/>
+      <c r="D373" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E373" s="31" t="inlineStr">
+        <is>
+          <t>El sistema no permite valores negativos ni un valor pagado mayor que el total.</t>
+        </is>
+      </c>
+      <c r="F373" s="23" t="n"/>
+      <c r="G373" s="23" t="n"/>
     </row>
     <row r="374" ht="18" customHeight="1">
       <c r="A374" s="7" t="n"/>
-      <c r="D374" s="17" t="n"/>
+      <c r="B374" s="24" t="n"/>
+      <c r="C374" s="24" t="n"/>
+      <c r="D374" s="15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E374" s="31" t="inlineStr">
+        <is>
+          <t>El plan vigente del miembro es el último plan activo registrado.</t>
+        </is>
+      </c>
+      <c r="F374" s="24" t="n"/>
+      <c r="G374" s="24" t="n"/>
     </row>
     <row r="375" ht="18" customHeight="1">
       <c r="A375" s="7" t="n"/>
-      <c r="D375" s="17" t="n"/>
+      <c r="B375" s="34" t="n"/>
+      <c r="C375" s="34" t="n"/>
+      <c r="D375" s="35" t="n"/>
+      <c r="E375" s="34" t="n"/>
+      <c r="F375" s="34" t="n"/>
+      <c r="G375" s="34" t="n"/>
     </row>
     <row r="376" ht="18" customHeight="1">
       <c r="A376" s="7" t="n"/>
-      <c r="D376" s="17" t="n"/>
+      <c r="B376" s="25" t="inlineStr">
+        <is>
+          <t>HU-63: Eliminar la cuenta del gimnasio y sus datos</t>
+        </is>
+      </c>
+      <c r="C376" s="28" t="inlineStr">
+        <is>
+          <t>Como dueño del gimnasio, quiero eliminar mi cuenta y todos los datos del gimnasio, para que pueda ejercer mi derecho de supresión de datos personales.</t>
+        </is>
+      </c>
+      <c r="D376" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E376" s="26" t="inlineStr">
+        <is>
+          <t>La opción está en la página de eliminación de cuenta y requiere sesión iniciada.</t>
+        </is>
+      </c>
+      <c r="F376" s="30" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G376" s="26" t="inlineStr">
+        <is>
+          <t>Operación DELETE de la cuenta del gimnasio en el módulo Cumplimiento (RQF-22). Relacionado con RQNF-12.</t>
+        </is>
+      </c>
     </row>
     <row r="377" ht="18" customHeight="1">
       <c r="A377" s="7" t="n"/>
-      <c r="D377" s="17" t="n"/>
+      <c r="B377" s="23" t="n"/>
+      <c r="C377" s="23" t="n"/>
+      <c r="D377" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E377" s="26" t="inlineStr">
+        <is>
+          <t>El sistema exige marcar una casilla de confirmación y permite indicar el motivo.</t>
+        </is>
+      </c>
+      <c r="F377" s="23" t="n"/>
+      <c r="G377" s="23" t="n"/>
     </row>
     <row r="378" ht="18" customHeight="1">
       <c r="A378" s="7" t="n"/>
-      <c r="D378" s="17" t="n"/>
+      <c r="B378" s="23" t="n"/>
+      <c r="C378" s="23" t="n"/>
+      <c r="D378" s="11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E378" s="26" t="inlineStr">
+        <is>
+          <t>Se eliminan en una sola transacción los miembros, asistencias, planes, mensajes, personal y el gimnasio.</t>
+        </is>
+      </c>
+      <c r="F378" s="23" t="n"/>
+      <c r="G378" s="23" t="n"/>
     </row>
     <row r="379" ht="18" customHeight="1">
       <c r="A379" s="7" t="n"/>
-      <c r="D379" s="17" t="n"/>
+      <c r="B379" s="23" t="n"/>
+      <c r="C379" s="23" t="n"/>
+      <c r="D379" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E379" s="26" t="inlineStr">
+        <is>
+          <t>Si la eliminación falla, no se borra nada (la transacción se revierte).</t>
+        </is>
+      </c>
+      <c r="F379" s="23" t="n"/>
+      <c r="G379" s="23" t="n"/>
     </row>
     <row r="380" ht="18" customHeight="1">
       <c r="A380" s="7" t="n"/>
-      <c r="D380" s="17" t="n"/>
+      <c r="B380" s="24" t="n"/>
+      <c r="C380" s="24" t="n"/>
+      <c r="D380" s="11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E380" s="26" t="inlineStr">
+        <is>
+          <t>Al terminar, la sesión se cierra y la cuenta ya no puede iniciar sesión.</t>
+        </is>
+      </c>
+      <c r="F380" s="24" t="n"/>
+      <c r="G380" s="24" t="n"/>
     </row>
     <row r="381" ht="18" customHeight="1">
       <c r="A381" s="7" t="n"/>
-      <c r="D381" s="17" t="n"/>
+      <c r="B381" s="34" t="n"/>
+      <c r="C381" s="34" t="n"/>
+      <c r="D381" s="35" t="n"/>
+      <c r="E381" s="34" t="n"/>
+      <c r="F381" s="34" t="n"/>
+      <c r="G381" s="34" t="n"/>
     </row>
     <row r="382" ht="18" customHeight="1">
       <c r="A382" s="7" t="n"/>
-      <c r="D382" s="17" t="n"/>
+      <c r="B382" s="27" t="inlineStr">
+        <is>
+          <t>HU-64: Ver avisos accionables en el centro de notificaciones</t>
+        </is>
+      </c>
+      <c r="C382" s="29" t="inlineStr">
+        <is>
+          <t>Como administrador o recepcionista, quiero ver en la campana del encabezado los miembros con membresía vencida, por vencer o en riesgo de abandono, para que pueda contactarlos a tiempo.</t>
+        </is>
+      </c>
+      <c r="D382" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E382" s="31" t="inlineStr">
+        <is>
+          <t>La campana está en todas las pantallas del panel y muestra cuántos avisos hay.</t>
+        </is>
+      </c>
+      <c r="F382" s="22" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G382" s="31" t="inlineStr">
+        <is>
+          <t>Operación READ del centro de notificaciones del módulo Dashboard (RQF-23). Relacionado con RQF-08 y RQF-09.</t>
+        </is>
+      </c>
     </row>
     <row r="383" ht="18" customHeight="1">
       <c r="A383" s="7" t="n"/>
-      <c r="D383" s="17" t="n"/>
+      <c r="B383" s="23" t="n"/>
+      <c r="C383" s="23" t="n"/>
+      <c r="D383" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E383" s="31" t="inlineStr">
+        <is>
+          <t>Los avisos se agrupan en membresías vencidas, por vencer y miembros en riesgo.</t>
+        </is>
+      </c>
+      <c r="F383" s="23" t="n"/>
+      <c r="G383" s="23" t="n"/>
     </row>
     <row r="384" ht="18" customHeight="1">
       <c r="A384" s="7" t="n"/>
-      <c r="D384" s="17" t="n"/>
+      <c r="B384" s="23" t="n"/>
+      <c r="C384" s="23" t="n"/>
+      <c r="D384" s="15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E384" s="31" t="inlineStr">
+        <is>
+          <t>Los días de anticipación y de inactividad salen de la configuración del gimnasio.</t>
+        </is>
+      </c>
+      <c r="F384" s="23" t="n"/>
+      <c r="G384" s="23" t="n"/>
     </row>
     <row r="385" ht="18" customHeight="1">
       <c r="A385" s="7" t="n"/>
-      <c r="D385" s="17" t="n"/>
+      <c r="B385" s="23" t="n"/>
+      <c r="C385" s="23" t="n"/>
+      <c r="D385" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E385" s="31" t="inlineStr">
+        <is>
+          <t>Desde cada aviso se abre WhatsApp con el mensaje listo para el miembro.</t>
+        </is>
+      </c>
+      <c r="F385" s="23" t="n"/>
+      <c r="G385" s="23" t="n"/>
     </row>
     <row r="386" ht="18" customHeight="1">
       <c r="A386" s="7" t="n"/>
-      <c r="D386" s="17" t="n"/>
+      <c r="B386" s="24" t="n"/>
+      <c r="C386" s="24" t="n"/>
+      <c r="D386" s="15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E386" s="31" t="inlineStr">
+        <is>
+          <t>Cada contacto queda registrado con fecha, canal y estado.</t>
+        </is>
+      </c>
+      <c r="F386" s="24" t="n"/>
+      <c r="G386" s="24" t="n"/>
     </row>
     <row r="387" ht="18" customHeight="1">
       <c r="A387" s="7" t="n"/>
-      <c r="D387" s="17" t="n"/>
+      <c r="B387" s="34" t="n"/>
+      <c r="C387" s="34" t="n"/>
+      <c r="D387" s="35" t="n"/>
+      <c r="E387" s="34" t="n"/>
+      <c r="F387" s="34" t="n"/>
+      <c r="G387" s="34" t="n"/>
     </row>
     <row r="388" ht="18" customHeight="1">
       <c r="A388" s="7" t="n"/>
-      <c r="D388" s="17" t="n"/>
+      <c r="B388" s="25" t="inlineStr">
+        <is>
+          <t>HU-65: Consultar la vista de miembros activos del gimnasio</t>
+        </is>
+      </c>
+      <c r="C388" s="28" t="inlineStr">
+        <is>
+          <t>Como administrador o recepcionista, quiero consultar un listado paginado de los miembros activos de mi gimnasio, para que pueda revisar rápidamente su plan y su vigencia.</t>
+        </is>
+      </c>
+      <c r="D388" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E388" s="26" t="inlineStr">
+        <is>
+          <t>El listado muestra nombre, documento, contacto, plan y fechas de vigencia, sin el identificador interno.</t>
+        </is>
+      </c>
+      <c r="F388" s="30" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G388" s="26" t="inlineStr">
+        <is>
+          <t>Operación READ de la vista de miembros activos en el módulo Gestión de Miembros (RQF-25). Relacionado con RQNF-05.</t>
+        </is>
+      </c>
     </row>
     <row r="389" ht="18" customHeight="1">
       <c r="A389" s="7" t="n"/>
-      <c r="D389" s="17" t="n"/>
+      <c r="B389" s="23" t="n"/>
+      <c r="C389" s="23" t="n"/>
+      <c r="D389" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E389" s="26" t="inlineStr">
+        <is>
+          <t>Solo aparecen miembros de mi gimnasio.</t>
+        </is>
+      </c>
+      <c r="F389" s="23" t="n"/>
+      <c r="G389" s="23" t="n"/>
     </row>
     <row r="390" ht="18" customHeight="1">
       <c r="A390" s="7" t="n"/>
-      <c r="D390" s="17" t="n"/>
+      <c r="B390" s="23" t="n"/>
+      <c r="C390" s="23" t="n"/>
+      <c r="D390" s="11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E390" s="26" t="inlineStr">
+        <is>
+          <t>Solo el personal del gimnasio puede consultarlo; un miembro desde la app no tiene acceso.</t>
+        </is>
+      </c>
+      <c r="F390" s="23" t="n"/>
+      <c r="G390" s="23" t="n"/>
     </row>
     <row r="391" ht="18" customHeight="1">
       <c r="A391" s="7" t="n"/>
-      <c r="D391" s="17" t="n"/>
+      <c r="B391" s="23" t="n"/>
+      <c r="C391" s="23" t="n"/>
+      <c r="D391" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E391" s="26" t="inlineStr">
+        <is>
+          <t>El listado se puede paginar.</t>
+        </is>
+      </c>
+      <c r="F391" s="23" t="n"/>
+      <c r="G391" s="23" t="n"/>
     </row>
     <row r="392" ht="18" customHeight="1">
       <c r="A392" s="7" t="n"/>
-      <c r="D392" s="17" t="n"/>
+      <c r="B392" s="24" t="n"/>
+      <c r="C392" s="24" t="n"/>
+      <c r="D392" s="11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E392" s="26" t="inlineStr">
+        <is>
+          <t>La vista que lo alimenta se crea con las migraciones del sistema y usa el plan vigente de cada miembro.</t>
+        </is>
+      </c>
+      <c r="F392" s="24" t="n"/>
+      <c r="G392" s="24" t="n"/>
     </row>
     <row r="393" ht="18" customHeight="1">
       <c r="A393" s="7" t="n"/>
-      <c r="D393" s="17" t="n"/>
+      <c r="B393" s="34" t="n"/>
+      <c r="C393" s="34" t="n"/>
+      <c r="D393" s="35" t="n"/>
+      <c r="E393" s="34" t="n"/>
+      <c r="F393" s="34" t="n"/>
+      <c r="G393" s="34" t="n"/>
     </row>
     <row r="394" ht="18" customHeight="1">
       <c r="A394" s="7" t="n"/>
-      <c r="D394" s="17" t="n"/>
+      <c r="B394" s="27" t="inlineStr">
+        <is>
+          <t>HU-66: Editar mi perfil desde la app móvil</t>
+        </is>
+      </c>
+      <c r="C394" s="29" t="inlineStr">
+        <is>
+          <t>Como miembro, quiero actualizar mi teléfono, mi correo y mi contacto de emergencia desde la app, para que el gimnasio tenga mis datos al día.</t>
+        </is>
+      </c>
+      <c r="D394" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E394" s="31" t="inlineStr">
+        <is>
+          <t>La app tiene una pantalla para editar el perfil.</t>
+        </is>
+      </c>
+      <c r="F394" s="22" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G394" s="31" t="inlineStr">
+        <is>
+          <t>Operación UPDATE del perfil en el módulo App del miembro (RQF-26). Depende de HU-57.</t>
+        </is>
+      </c>
     </row>
     <row r="395" ht="18" customHeight="1">
       <c r="A395" s="7" t="n"/>
-      <c r="D395" s="17" t="n"/>
+      <c r="B395" s="23" t="n"/>
+      <c r="C395" s="23" t="n"/>
+      <c r="D395" s="15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E395" s="31" t="inlineStr">
+        <is>
+          <t>Puedo cambiar mi teléfono, mi correo y mi contacto de emergencia.</t>
+        </is>
+      </c>
+      <c r="F395" s="23" t="n"/>
+      <c r="G395" s="23" t="n"/>
     </row>
     <row r="396" ht="18" customHeight="1">
       <c r="A396" s="7" t="n"/>
-      <c r="D396" s="17" t="n"/>
+      <c r="B396" s="23" t="n"/>
+      <c r="C396" s="23" t="n"/>
+      <c r="D396" s="15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E396" s="31" t="inlineStr">
+        <is>
+          <t>Los cambios se guardan solo en mi propio perfil.</t>
+        </is>
+      </c>
+      <c r="F396" s="23" t="n"/>
+      <c r="G396" s="23" t="n"/>
     </row>
     <row r="397" ht="18" customHeight="1">
       <c r="A397" s="7" t="n"/>
-      <c r="D397" s="17" t="n"/>
+      <c r="B397" s="23" t="n"/>
+      <c r="C397" s="23" t="n"/>
+      <c r="D397" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E397" s="31" t="inlineStr">
+        <is>
+          <t>El sistema rechaza un correo que ya use otro miembro del gimnasio.</t>
+        </is>
+      </c>
+      <c r="F397" s="23" t="n"/>
+      <c r="G397" s="23" t="n"/>
     </row>
     <row r="398" ht="18" customHeight="1">
       <c r="A398" s="7" t="n"/>
-      <c r="D398" s="17" t="n"/>
+      <c r="B398" s="24" t="n"/>
+      <c r="C398" s="24" t="n"/>
+      <c r="D398" s="15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E398" s="31" t="inlineStr">
+        <is>
+          <t>Al guardar, la app muestra los datos actualizados.</t>
+        </is>
+      </c>
+      <c r="F398" s="24" t="n"/>
+      <c r="G398" s="24" t="n"/>
     </row>
     <row r="399" ht="18" customHeight="1">
       <c r="A399" s="7" t="n"/>
-      <c r="D399" s="17" t="n"/>
+      <c r="B399" s="34" t="n"/>
+      <c r="C399" s="34" t="n"/>
+      <c r="D399" s="35" t="n"/>
+      <c r="E399" s="34" t="n"/>
+      <c r="F399" s="34" t="n"/>
+      <c r="G399" s="34" t="n"/>
     </row>
     <row r="400" ht="18" customHeight="1">
       <c r="A400" s="7" t="n"/>
@@ -9496,16 +10184,19 @@
       <c r="D996" s="17" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="233">
+  <mergeCells count="265">
+    <mergeCell ref="C394:C398"/>
     <mergeCell ref="F106:F110"/>
     <mergeCell ref="B88:B92"/>
     <mergeCell ref="G196:G200"/>
     <mergeCell ref="B82:B86"/>
     <mergeCell ref="C232:C236"/>
+    <mergeCell ref="B358:B362"/>
     <mergeCell ref="G64:G68"/>
     <mergeCell ref="C46:C50"/>
     <mergeCell ref="C178:C182"/>
     <mergeCell ref="B124:B128"/>
+    <mergeCell ref="B388:B392"/>
     <mergeCell ref="C70:C74"/>
     <mergeCell ref="B256:B260"/>
     <mergeCell ref="F220:F224"/>
@@ -9520,9 +10211,12 @@
     <mergeCell ref="B334:B338"/>
     <mergeCell ref="G40:G44"/>
     <mergeCell ref="G226:G230"/>
+    <mergeCell ref="G364:G368"/>
     <mergeCell ref="G106:G110"/>
+    <mergeCell ref="F376:F380"/>
     <mergeCell ref="B190:B194"/>
     <mergeCell ref="F166:F170"/>
+    <mergeCell ref="G382:G386"/>
     <mergeCell ref="C154:C158"/>
     <mergeCell ref="B100:B104"/>
     <mergeCell ref="B280:B284"/>
@@ -9542,6 +10236,7 @@
     <mergeCell ref="B322:B326"/>
     <mergeCell ref="F232:F236"/>
     <mergeCell ref="F316:F320"/>
+    <mergeCell ref="F394:F398"/>
     <mergeCell ref="F298:F302"/>
     <mergeCell ref="C118:C122"/>
     <mergeCell ref="G82:G86"/>
@@ -9550,6 +10245,7 @@
     <mergeCell ref="C10:C14"/>
     <mergeCell ref="C16:C20"/>
     <mergeCell ref="B244:B248"/>
+    <mergeCell ref="G358:G362"/>
     <mergeCell ref="B136:B140"/>
     <mergeCell ref="B70:B74"/>
     <mergeCell ref="F160:F164"/>
@@ -9562,12 +10258,15 @@
     <mergeCell ref="G34:G38"/>
     <mergeCell ref="C52:C56"/>
     <mergeCell ref="B178:B182"/>
+    <mergeCell ref="F382:F386"/>
     <mergeCell ref="G4:G8"/>
     <mergeCell ref="F274:F278"/>
     <mergeCell ref="B310:B314"/>
     <mergeCell ref="F130:F134"/>
     <mergeCell ref="B226:B230"/>
     <mergeCell ref="G334:G338"/>
+    <mergeCell ref="C370:C374"/>
+    <mergeCell ref="C352:C356"/>
     <mergeCell ref="F58:F62"/>
     <mergeCell ref="C328:C332"/>
     <mergeCell ref="C262:C266"/>
@@ -9583,10 +10282,13 @@
     <mergeCell ref="C304:C308"/>
     <mergeCell ref="B154:B158"/>
     <mergeCell ref="G22:G26"/>
+    <mergeCell ref="F358:F362"/>
     <mergeCell ref="G202:G206"/>
+    <mergeCell ref="F352:F356"/>
     <mergeCell ref="F148:F152"/>
     <mergeCell ref="B286:B290"/>
     <mergeCell ref="G316:G320"/>
+    <mergeCell ref="C376:C380"/>
     <mergeCell ref="F118:F122"/>
     <mergeCell ref="C184:C188"/>
     <mergeCell ref="G208:G212"/>
@@ -9617,12 +10319,18 @@
     <mergeCell ref="G184:G188"/>
     <mergeCell ref="G310:G314"/>
     <mergeCell ref="B166:B170"/>
+    <mergeCell ref="C364:C368"/>
+    <mergeCell ref="F370:F374"/>
+    <mergeCell ref="B376:B380"/>
     <mergeCell ref="G58:G62"/>
     <mergeCell ref="G220:G224"/>
     <mergeCell ref="B298:B302"/>
     <mergeCell ref="C148:C152"/>
     <mergeCell ref="F262:F266"/>
+    <mergeCell ref="B364:B368"/>
+    <mergeCell ref="C388:C392"/>
     <mergeCell ref="F184:F188"/>
+    <mergeCell ref="G388:G392"/>
     <mergeCell ref="B112:B116"/>
     <mergeCell ref="B274:B278"/>
     <mergeCell ref="F46:F50"/>
@@ -9638,15 +10346,18 @@
     <mergeCell ref="B268:B272"/>
     <mergeCell ref="F346:F350"/>
     <mergeCell ref="G76:G80"/>
+    <mergeCell ref="C358:C362"/>
     <mergeCell ref="F250:F254"/>
     <mergeCell ref="B160:B164"/>
     <mergeCell ref="B340:B344"/>
+    <mergeCell ref="G370:G374"/>
     <mergeCell ref="F172:F176"/>
     <mergeCell ref="F4:F8"/>
     <mergeCell ref="C34:C38"/>
     <mergeCell ref="G238:G242"/>
     <mergeCell ref="B106:B110"/>
     <mergeCell ref="G232:G236"/>
+    <mergeCell ref="B382:B386"/>
     <mergeCell ref="C166:C170"/>
     <mergeCell ref="C160:C164"/>
     <mergeCell ref="C4:C8"/>
@@ -9663,6 +10374,7 @@
     <mergeCell ref="F16:F20"/>
     <mergeCell ref="B52:B56"/>
     <mergeCell ref="G346:G350"/>
+    <mergeCell ref="C382:C386"/>
     <mergeCell ref="C100:C104"/>
     <mergeCell ref="F292:F296"/>
     <mergeCell ref="B328:B332"/>
@@ -9678,11 +10390,13 @@
     <mergeCell ref="C202:C206"/>
     <mergeCell ref="G148:G152"/>
     <mergeCell ref="B148:B152"/>
+    <mergeCell ref="B352:B356"/>
     <mergeCell ref="C40:C44"/>
     <mergeCell ref="F190:F194"/>
     <mergeCell ref="B250:B254"/>
     <mergeCell ref="C316:C320"/>
     <mergeCell ref="C76:C80"/>
+    <mergeCell ref="G394:G398"/>
     <mergeCell ref="F100:F104"/>
     <mergeCell ref="B118:B122"/>
     <mergeCell ref="G250:G254"/>
@@ -9698,6 +10412,7 @@
     <mergeCell ref="F136:F140"/>
     <mergeCell ref="B196:B200"/>
     <mergeCell ref="G88:G92"/>
+    <mergeCell ref="B394:B398"/>
     <mergeCell ref="F64:F68"/>
     <mergeCell ref="C292:C296"/>
     <mergeCell ref="B142:B146"/>
@@ -9706,13 +10421,16 @@
     <mergeCell ref="G286:G290"/>
     <mergeCell ref="G130:G134"/>
     <mergeCell ref="B16:B20"/>
+    <mergeCell ref="B370:B374"/>
     <mergeCell ref="C58:C62"/>
     <mergeCell ref="C220:C224"/>
     <mergeCell ref="F10:F14"/>
     <mergeCell ref="G214:G218"/>
+    <mergeCell ref="F364:F368"/>
     <mergeCell ref="G52:G56"/>
     <mergeCell ref="B184:B188"/>
     <mergeCell ref="F256:F260"/>
+    <mergeCell ref="F388:F392"/>
     <mergeCell ref="G328:G332"/>
     <mergeCell ref="F178:F182"/>
     <mergeCell ref="F280:F284"/>
@@ -9720,10 +10438,12 @@
     <mergeCell ref="B208:B212"/>
     <mergeCell ref="F310:F314"/>
     <mergeCell ref="F202:F206"/>
+    <mergeCell ref="G352:G356"/>
     <mergeCell ref="G262:G266"/>
     <mergeCell ref="C142:C146"/>
     <mergeCell ref="B346:B350"/>
     <mergeCell ref="G118:G122"/>
+    <mergeCell ref="G376:G380"/>
     <mergeCell ref="C112:C116"/>
     <mergeCell ref="F244:F248"/>
     <mergeCell ref="G28:G32"/>
@@ -9743,7 +10463,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F4 F10 F16 F22 F28 F34 F40 F46 F52 F58 F64 F70 F76 F82 F88 F94 F100 F106 F112 F118 F124 F130 F136 F142 F148 F154 F160 F166 F172 F178 F184 F190 F196 F202 F208 F214 F220 F226 F232 F238 F244 F250 F256 F262 F268 F274 F280 F286 F292 F298 F304 F310 F316 F322 F328 F334 F340 F346" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F4 F10 F16 F22 F28 F34 F40 F46 F52 F58 F64 F70 F76 F82 F88 F94 F100 F106 F112 F118 F124 F130 F136 F142 F148 F154 F160 F166 F172 F178 F184 F190 F196 F202 F208 F214 F220 F226 F232 F238 F244 F250 F256 F262 F268 F274 F280 F286 F292 F298 F304 F310 F316 F322 F328 F334 F340 F346 F352 F358 F364 F370 F376 F382 F388 F394" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>'Prioridad - No borrar'!$B$3:$B$5</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(historias): reasigna las HU de los requisitos retirados
Por decision de Luis se retiran RQF-23..25 y RQF-26 se fusiona en RQF-15.
Las historias se conservan y cambian de requisito: HU-64 pasa a RQF-08,
HU-65 a RQF-03 y HU-66 a RQF-15; HU-34 vuelve a RQF-05 y RQF-07.
</commit_message>
<xml_diff>
--- a/Documentación/Plantilla historias de usuario.xlsx
+++ b/Documentación/Plantilla historias de usuario.xlsx
@@ -4492,7 +4492,7 @@
       </c>
       <c r="G202" s="31" t="inlineStr">
         <is>
-          <t>Operación READ en tiempo real del módulo Check-in (RQF-05, RQF-07 y RQF-24).</t>
+          <t>Operación READ en tiempo real del módulo Check-in (RQF-05 y RQF-07).</t>
         </is>
       </c>
     </row>
@@ -7494,7 +7494,7 @@
       </c>
       <c r="G382" s="31" t="inlineStr">
         <is>
-          <t>Operación READ del centro de notificaciones del módulo Dashboard (RQF-23). Relacionado con RQF-08 y RQF-09.</t>
+          <t>Operación READ del centro de notificaciones en el módulo Alertas de Abandono (RQF-08). Relacionado con RQF-04 y RQF-09.</t>
         </is>
       </c>
     </row>
@@ -7604,7 +7604,7 @@
       </c>
       <c r="G388" s="26" t="inlineStr">
         <is>
-          <t>Operación READ de la vista de miembros activos en el módulo Gestión de Miembros (RQF-25). Relacionado con RQNF-05.</t>
+          <t>Operación READ de la vista de miembros activos en el módulo Gestión de Miembros (RQF-03). Relacionado con RQNF-05.</t>
         </is>
       </c>
     </row>
@@ -7714,7 +7714,7 @@
       </c>
       <c r="G394" s="31" t="inlineStr">
         <is>
-          <t>Operación UPDATE del perfil en el módulo App del miembro (RQF-26). Depende de HU-57.</t>
+          <t>Operación UPDATE del perfil en el módulo App del miembro (RQF-15). Depende de HU-57.</t>
         </is>
       </c>
     </row>

</xml_diff>